<commit_message>
Reskin do dashboard para tema Fluxo + setup de deploy
Aplica identidade visual da Fluxo (preto + laranja) no dashboard e adiciona
arquivos de configuração para publicação no Streamlit Community Cloud
(requirements.txt, .streamlit/config.toml, .gitignore, DEPLOY.md).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipefy-crm/dados/relatorio_completo.xlsx
+++ b/pipefy-crm/dados/relatorio_completo.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Objeções" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Por Responsável" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Por Fase" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objeções" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Responsável" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por Fase" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -465,19 +465,19 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>510</v>
+        <v>737</v>
       </c>
       <c r="D2" t="n">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="E2" t="n">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="F2" t="n">
-        <v>615</v>
+        <v>903</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="3">
@@ -487,22 +487,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C3" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="D3" t="n">
         <v>19</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="G3" t="n">
-        <v>46.1</v>
+        <v>44.4</v>
       </c>
     </row>
     <row r="4">
@@ -512,22 +512,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="G4" t="n">
-        <v>15.4</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="5">
@@ -540,144 +540,144 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G5" t="n">
-        <v>12.5</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sim, prazo</t>
+          <t>Sim, outros</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
+        <v>23</v>
+      </c>
+      <c r="G6" t="n">
         <v>13</v>
-      </c>
-      <c r="G6" t="n">
-        <v>15.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Sim, validade</t>
+          <t>Sim, prazo</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G7" t="n">
-        <v>15.4</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sim, outros</t>
+          <t>Sim, validade</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="n">
+        <v>6</v>
+      </c>
+      <c r="D8" t="n">
         <v>5</v>
       </c>
-      <c r="D8" t="n">
-        <v>4</v>
-      </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G8" t="n">
-        <v>9.1</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sim, autoridade</t>
+          <t>Sim, parcelamento</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G9" t="n">
-        <v>12.5</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sim, parcelamento</t>
+          <t>Sim, autoridade</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G10" t="n">
-        <v>37.5</v>
+        <v>11.1</v>
       </c>
     </row>
   </sheetData>
@@ -691,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -738,22 +738,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C2" t="n">
-        <v>173</v>
+        <v>248</v>
       </c>
       <c r="D2" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>221</v>
+        <v>300</v>
       </c>
       <c r="G2" t="n">
-        <v>7.2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -766,13 +766,13 @@
         <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D3" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>165</v>
@@ -784,51 +784,51 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Enrico Cardoso</t>
+          <t>Estela Vianna</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="D4" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G4" t="n">
-        <v>3.1</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Estela Vianna</t>
+          <t>Enrico Cardoso</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D5" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="G5" t="n">
-        <v>2.2</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="6">
@@ -838,569 +838,569 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C6" t="n">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G6" t="n">
-        <v>9.199999999999999</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gabriela Boechat</t>
+          <t>Jonas Pimenta</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C7" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D7" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="F7" t="n">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="G7" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rodrigo Polly Anthés</t>
+          <t>IGOR SILVA MONIZ</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="D8" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="G8" t="n">
-        <v>11.5</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IGOR SILVA MONIZ</t>
+          <t>Ana Clara Belmonte Garcia</t>
         </is>
       </c>
       <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>66</v>
+      </c>
+      <c r="D9" t="n">
         <v>6</v>
       </c>
-      <c r="C9" t="n">
-        <v>65</v>
-      </c>
-      <c r="D9" t="n">
-        <v>13</v>
-      </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F9" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G9" t="n">
-        <v>7.1</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Marcos Paulo Santos</t>
+          <t>Gabriela Boechat</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C10" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="D10" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="G10" t="n">
-        <v>6.8</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Elizeu dos Santos Coelho</t>
+          <t>Rodrigo Polly Anthés</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C11" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D11" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="G11" t="n">
-        <v>7.2</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Lucas Pimenta</t>
+          <t>Marcos Paulo Santos</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C12" t="n">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="G12" t="n">
-        <v>3.1</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jonas Pimenta</t>
+          <t>Elizeu dos Santos Coelho</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="D13" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="G13" t="n">
-        <v>10.7</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gabriel Saldanha</t>
+          <t>Lucas Pimenta</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="G14" t="n">
-        <v>9.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gabriela Andrade</t>
+          <t>Miguel Mendes Louzada de Souza</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" t="n">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="D15" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" t="n">
         <v>11</v>
       </c>
-      <c r="E15" t="n">
-        <v>7</v>
-      </c>
       <c r="F15" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="G15" t="n">
-        <v>11.4</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Beatriz Assunção</t>
+          <t>Gabriel Saldanha</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C16" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="G16" t="n">
-        <v>8.300000000000001</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Pedro Carneiro Cavalcante</t>
+          <t>Manuella Heringer Rocha Verbicaro Ramos</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F17" t="n">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="G17" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Emmanuel</t>
+          <t>Gabriela Andrade</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C18" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G18" t="n">
-        <v>5.9</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rafael Luiz Santos Nobre</t>
+          <t>Camilla Ribeiro Ferreira</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F19" t="n">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="G19" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gabriel Sanhudo Soares</t>
+          <t>Lucas Siqueira Vieira</t>
         </is>
       </c>
       <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>35</v>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" t="n">
         <v>9</v>
       </c>
-      <c r="C20" t="n">
-        <v>12</v>
-      </c>
-      <c r="D20" t="n">
-        <v>10</v>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
       <c r="F20" t="n">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="G20" t="n">
-        <v>28.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Maria Vitória Gomes Martins</t>
+          <t>Emmanuel</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>2</v>
       </c>
       <c r="C21" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D21" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="G21" t="n">
-        <v>8.699999999999999</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Davison Dhiego de Farias Mazzei</t>
+          <t>Beatriz Assunção</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="G22" t="n">
-        <v>13.3</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gabriela D’Agostini Fraga</t>
+          <t>Rafael Luiz Santos Nobre</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="D23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="G23" t="n">
-        <v>7.1</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Matheus Xavier Martins</t>
+          <t>Pedro Carneiro Cavalcante</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C24" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gabriel Pereira</t>
+          <t>Gabriel Sanhudo Soares</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D25" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G25" t="n">
-        <v>33.3</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Enzo Antunes Marmello</t>
+          <t>Guilherme Vanni de Lima Cavalcanti Wanderley</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="G26" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Manuella Heringer Rocha Verbicaro Ramos</t>
+          <t>Maria Vitória Gomes Martins</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="G27" t="n">
-        <v>0</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>marcos.paulo</t>
+          <t>Matheus Xavier Martins</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>0</v>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1409,39 +1409,39 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Camilla Ribeiro Ferreira</t>
+          <t>Erik Branco Queiroz</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>wallisonpereira-20221-poli</t>
+          <t>Davison Dhiego de Farias Mazzei</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>2</v>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -1450,132 +1450,132 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G30" t="n">
-        <v>40</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>natalia-rodrigues-poli</t>
+          <t>Gabriela D’Agostini Fraga</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pedro de Souza Angelo</t>
+          <t>Lucas Villaça</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F32" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G32" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Gilson Batista Machado Martins</t>
+          <t>Gabriel Pereira</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G33" t="n">
-        <v>25</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ana Clara Belmonte Garcia</t>
+          <t>Paulo Vitor Couto</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G34" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Stella Monteiro</t>
+          <t>Heitor Mendes</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>0</v>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1584,123 +1584,123 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cecília Nogueira Rosa</t>
+          <t>Enzo Antunes Marmello</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G36" t="n">
-        <v>33.3</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Eduardo Caldas</t>
+          <t>marcos.paulo</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G37" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Erik Branco Queiroz</t>
+          <t>Pedro de Souza Angelo</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Eduarda Braun Monteiro da Silva</t>
+          <t>Gilson Batista Machado Martins</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Lucas Siqueira Vieira</t>
+          <t>natalia-rodrigues-poli</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>0</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -1709,14 +1709,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mariana Fonseca</t>
+          <t>wallisonpereira-20221-poli</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
@@ -1725,57 +1725,57 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>João Victor Moraes</t>
+          <t>Eduarda Braun Monteiro da Silva</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C42" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Miguel Mendes Louzada de Souza</t>
+          <t>Renato Saboia</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>0</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G43" t="n">
         <v>0</v>
@@ -1784,64 +1784,64 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LUCAS CORDEIRO QUIRINO</t>
+          <t>Cecília Nogueira Rosa</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Guilherme Lameck</t>
+          <t>Vitor Malfa</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D45" t="n">
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Heitor Ferreira</t>
+          <t>Stella Monteiro</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>0</v>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
         <v>1</v>
@@ -1850,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
@@ -1859,7 +1859,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rafael Gondim</t>
+          <t>João Victor Moraes</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1869,26 +1869,26 @@
         <v>0</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G47" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Paulo Vitor Couto</t>
+          <t>Eduardo Caldas</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C48" t="n">
         <v>0</v>
@@ -1897,23 +1897,23 @@
         <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Nicollas Viellas Lee</t>
+          <t>Lucas Angelo Ribeiro</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C49" t="n">
         <v>0</v>
@@ -1922,35 +1922,35 @@
         <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G49" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>leonardorussosalles</t>
+          <t>Sem responsável</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>0</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G50" t="n">
         <v>0</v>
@@ -1959,23 +1959,23 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Vitor Malfa</t>
+          <t>Mariana Fonseca</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>0</v>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D51" t="n">
         <v>0</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G51" t="n">
         <v>0</v>
@@ -1984,17 +1984,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Sem responsável</t>
+          <t>Arthur Catelani Gomes da Silva</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C52" t="n">
         <v>0</v>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
@@ -2003,31 +2003,206 @@
         <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>Heitor Ferreira</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Guilherme Lameck</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Nicollas Viellas Lee</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>LUCAS CORDEIRO QUIRINO</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Rafael Gondim</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ericheubel-20241</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>leonardorussosalles</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>liviamonteiro-poli</t>
         </is>
       </c>
-      <c r="B53" t="n">
-        <v>0</v>
-      </c>
-      <c r="C53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" t="n">
-        <v>0</v>
-      </c>
-      <c r="E53" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" t="n">
+      <c r="B60" t="n">
+        <v>0</v>
+      </c>
+      <c r="C60" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2042,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2059,7 +2234,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -2067,12 +2242,12 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>575</v>
+        <v>838</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -2080,12 +2255,12 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>126</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -2093,25 +2268,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>56</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4. Dignóstico feito</t>
+          <t>2. Contato aberto</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -2119,25 +2294,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6. Proposta comercial feita</t>
+          <t>4. Diagnóstico feito</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -2145,33 +2320,46 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>5. Precificação/Aprovação em andamento</t>
+          <t>6. Proposta comercial feita</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2. Contato aberto</t>
+          <t>5. Precificação/Aprovação em andamento</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1. Oportunidade</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>